<commit_message>
adiciona movimentacoes de entrada no estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F61C2B-9B2F-4D7A-B1DC-5F3D6BD19675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5D4D07-31BC-4F46-8FC4-B0329792809F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro" sheetId="1" r:id="rId1"/>
+    <sheet name="Entrada" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
   <si>
     <t>SKU</t>
   </si>
@@ -237,6 +238,33 @@
   </si>
   <si>
     <t>Hub expansor USB compacto</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Quantidade Entrada</t>
+  </si>
+  <si>
+    <t>Responsável</t>
+  </si>
+  <si>
+    <t>Observação</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Compra inicial</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Marcos</t>
+  </si>
+  <si>
+    <t>Reposição</t>
   </si>
 </sst>
 </file>
@@ -283,16 +311,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
@@ -320,9 +358,26 @@
     <tableColumn id="2" xr3:uid="{474B68BA-BE3F-4822-A13D-98B92741539B}" name="Produto"/>
     <tableColumn id="3" xr3:uid="{C9C1ED03-FCD0-490A-AE7B-3D65AB9EBFBB}" name="Descrição"/>
     <tableColumn id="4" xr3:uid="{8BEC5BD3-48D4-4690-B9D3-B90E65A45828}" name="Categoria"/>
-    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="4"/>
     <tableColumn id="6" xr3:uid="{EA58917D-0C34-4FB2-A614-DCAD68AA44F6}" name="Fornecedor"/>
-    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}" name="tbEntrada" displayName="tbEntrada" ref="A1:F26" totalsRowShown="0">
+  <autoFilter ref="A1:F26" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{7987F022-B4FC-4F00-B1FF-6BFCB106433D}" name="SKU"/>
+    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="1">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{575BEAB7-E3EC-442C-9D56-D43256ABCBFE}" name="Responsável"/>
+    <tableColumn id="6" xr3:uid="{3F64F76D-003F-4F5F-B825-2C63E0C4FEBC}" name="Observação"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1034,4 +1089,570 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8332FF2-8A94-48BE-8D82-D1718948A8B1}">
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="28.88671875" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="21.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46056</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Fone Bluetooth AirMax</v>
+      </c>
+      <c r="D2" s="4">
+        <v>80</v>
+      </c>
+      <c r="E2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>46056</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Caixa de Som MiniBass</v>
+      </c>
+      <c r="D3" s="4">
+        <v>60</v>
+      </c>
+      <c r="E3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>46057</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Mouse Gamer ProClick</v>
+      </c>
+      <c r="D4" s="4">
+        <v>100</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46057</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Teclado Mecânico KeyStorm</v>
+      </c>
+      <c r="D5" s="4">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Webcam Full HD VisionCam</v>
+      </c>
+      <c r="D6" s="4">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Carregador USB-C Turbo</v>
+      </c>
+      <c r="D7" s="4">
+        <v>120</v>
+      </c>
+      <c r="E7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46059</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Cabo USB-C Reforçado</v>
+      </c>
+      <c r="D8" s="4">
+        <v>200</v>
+      </c>
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46059</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Power Bank 10000mAh</v>
+      </c>
+      <c r="D9" s="4">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46060</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Luminária LED Smart</v>
+      </c>
+      <c r="D10" s="4">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>46060</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Tomada Inteligente Wi-Fi</v>
+      </c>
+      <c r="D11" s="4">
+        <v>65</v>
+      </c>
+      <c r="E11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>46061</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Roteador Wi-Fi Dual Band</v>
+      </c>
+      <c r="D12" s="4">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>46061</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Repetidor de Sinal Wi-Fi</v>
+      </c>
+      <c r="D13" s="4">
+        <v>75</v>
+      </c>
+      <c r="E13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>SSD 480GB FastDisk</v>
+      </c>
+      <c r="D14" s="4">
+        <v>90</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Pendrive 64GB DataGo</v>
+      </c>
+      <c r="D15" s="4">
+        <v>150</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>46063</v>
+      </c>
+      <c r="B16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Hub USB 4 Portas</v>
+      </c>
+      <c r="D16" s="4">
+        <v>110</v>
+      </c>
+      <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Fone Bluetooth AirMax</v>
+      </c>
+      <c r="D17" s="4">
+        <v>30</v>
+      </c>
+      <c r="E17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Carregador USB-C Turbo</v>
+      </c>
+      <c r="D18" s="4">
+        <v>50</v>
+      </c>
+      <c r="E18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>46071</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Cabo USB-C Reforçado</v>
+      </c>
+      <c r="D19" s="4">
+        <v>100</v>
+      </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>46071</v>
+      </c>
+      <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>SSD 480GB FastDisk</v>
+      </c>
+      <c r="D20" s="4">
+        <v>40</v>
+      </c>
+      <c r="E20" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>46073</v>
+      </c>
+      <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Pendrive 64GB DataGo</v>
+      </c>
+      <c r="D21" s="4">
+        <v>80</v>
+      </c>
+      <c r="E21" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>46074</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Mouse Gamer ProClick</v>
+      </c>
+      <c r="D22" s="4">
+        <v>35</v>
+      </c>
+      <c r="E22" t="s">
+        <v>72</v>
+      </c>
+      <c r="F22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>46075</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Tomada Inteligente Wi-Fi</v>
+      </c>
+      <c r="D23" s="4">
+        <v>25</v>
+      </c>
+      <c r="E23" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Repetidor de Sinal Wi-Fi</v>
+      </c>
+      <c r="D24" s="4">
+        <v>30</v>
+      </c>
+      <c r="E24" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>46077</v>
+      </c>
+      <c r="B25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Hub USB 4 Portas</v>
+      </c>
+      <c r="D25" s="4">
+        <v>45</v>
+      </c>
+      <c r="E25" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>46078</v>
+      </c>
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" t="str">
+        <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Power Bank 10000mAh</v>
+      </c>
+      <c r="D26" s="4">
+        <v>20</v>
+      </c>
+      <c r="E26" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
adiciona movimentacoes de saida no estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5D4D07-31BC-4F46-8FC4-B0329792809F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C36FD7-61D8-4E87-B3D6-2253019FCA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro" sheetId="1" r:id="rId1"/>
     <sheet name="Entrada" sheetId="2" r:id="rId2"/>
+    <sheet name="Saída" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="82">
   <si>
     <t>SKU</t>
   </si>
@@ -265,6 +266,27 @@
   </si>
   <si>
     <t>Reposição</t>
+  </si>
+  <si>
+    <t>Quantidade Saída</t>
+  </si>
+  <si>
+    <t>Canal de Venda</t>
+  </si>
+  <si>
+    <t>Loja Física</t>
+  </si>
+  <si>
+    <t>Venda normal</t>
+  </si>
+  <si>
+    <t>Marketplace</t>
+  </si>
+  <si>
+    <t>Venda online</t>
+  </si>
+  <si>
+    <t>Campanha promocional</t>
   </si>
 </sst>
 </file>
@@ -321,7 +343,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="8">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -358,9 +389,9 @@
     <tableColumn id="2" xr3:uid="{474B68BA-BE3F-4822-A13D-98B92741539B}" name="Produto"/>
     <tableColumn id="3" xr3:uid="{C9C1ED03-FCD0-490A-AE7B-3D65AB9EBFBB}" name="Descrição"/>
     <tableColumn id="4" xr3:uid="{8BEC5BD3-48D4-4690-B9D3-B90E65A45828}" name="Categoria"/>
-    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="7"/>
     <tableColumn id="6" xr3:uid="{EA58917D-0C34-4FB2-A614-DCAD68AA44F6}" name="Fornecedor"/>
-    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -370,14 +401,29 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}" name="tbEntrada" displayName="tbEntrada" ref="A1:F26" totalsRowShown="0">
   <autoFilter ref="A1:F26" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{7987F022-B4FC-4F00-B1FF-6BFCB106433D}" name="SKU"/>
-    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{575BEAB7-E3EC-442C-9D56-D43256ABCBFE}" name="Responsável"/>
     <tableColumn id="6" xr3:uid="{3F64F76D-003F-4F5F-B825-2C63E0C4FEBC}" name="Observação"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}" name="tbSaida" displayName="tbSaida" ref="A1:F31" totalsRowShown="0">
+  <autoFilter ref="A1:F31" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{84870D34-BE9F-4CFC-A62B-6EE2B5631FD5}" name="Data" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{73BFB05B-0638-42FE-83E0-AB0F3445B4FF}" name="SKU"/>
+    <tableColumn id="3" xr3:uid="{63B5D954-F021-49FF-BBD4-26F9DF540E6B}" name="Produto" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{C7872616-E7BA-4C77-8D41-2068067BB2A7}" name="Quantidade Saída" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{9B35AB08-6C54-43E0-B34D-15830AD4E19C}" name="Canal de Venda"/>
+    <tableColumn id="6" xr3:uid="{AB3D24CB-C511-41D2-9E6C-DBF4DB411643}" name="Observação"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1655,4 +1701,672 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA5AD9DB-6B87-4ADF-B6B1-7040B728B6B2}">
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" customWidth="1"/>
+    <col min="4" max="4" width="26.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="24.21875" customWidth="1"/>
+    <col min="6" max="6" width="26.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46059</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>46059</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>46060</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="4">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46060</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46061</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46061</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4">
+        <v>35</v>
+      </c>
+      <c r="E7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Cabo USB-C Reforçado</v>
+      </c>
+      <c r="D8" s="4">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Power Bank 10000mAh</v>
+      </c>
+      <c r="D9" s="4">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46063</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Luminária LED Smart</v>
+      </c>
+      <c r="D10" s="4">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>46063</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Tomada Inteligente Wi-Fi</v>
+      </c>
+      <c r="D11" s="4">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>46064</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Roteador Wi-Fi Dual Band</v>
+      </c>
+      <c r="D12" s="4">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>46064</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Repetidor de Sinal Wi-Fi</v>
+      </c>
+      <c r="D13" s="4">
+        <v>22</v>
+      </c>
+      <c r="E13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>46065</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>SSD 480GB FastDisk</v>
+      </c>
+      <c r="D14" s="4">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>46065</v>
+      </c>
+      <c r="B15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Pendrive 64GB DataGo</v>
+      </c>
+      <c r="D15" s="4">
+        <v>60</v>
+      </c>
+      <c r="E15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>46066</v>
+      </c>
+      <c r="B16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Hub USB 4 Portas</v>
+      </c>
+      <c r="D16" s="4">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>46071</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Fone Bluetooth AirMax</v>
+      </c>
+      <c r="D17" s="4">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>46071</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Mouse Gamer ProClick</v>
+      </c>
+      <c r="D18" s="4">
+        <v>32</v>
+      </c>
+      <c r="E18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>46072</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Carregador USB-C Turbo</v>
+      </c>
+      <c r="D19" s="4">
+        <v>48</v>
+      </c>
+      <c r="E19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>46072</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Cabo USB-C Reforçado</v>
+      </c>
+      <c r="D20" s="4">
+        <v>95</v>
+      </c>
+      <c r="E20" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>46073</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>SSD 480GB FastDisk</v>
+      </c>
+      <c r="D21" s="4">
+        <v>42</v>
+      </c>
+      <c r="E21" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>46073</v>
+      </c>
+      <c r="B22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Pendrive 64GB DataGo</v>
+      </c>
+      <c r="D22" s="4">
+        <v>110</v>
+      </c>
+      <c r="E22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>46074</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Tomada Inteligente Wi-Fi</v>
+      </c>
+      <c r="D23" s="4">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>46075</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Repetidor de Sinal Wi-Fi</v>
+      </c>
+      <c r="D24" s="4">
+        <v>35</v>
+      </c>
+      <c r="E24" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Hub USB 4 Portas</v>
+      </c>
+      <c r="D25" s="4">
+        <v>50</v>
+      </c>
+      <c r="E25" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>46077</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Caixa de Som MiniBass</v>
+      </c>
+      <c r="D26" s="4">
+        <v>18</v>
+      </c>
+      <c r="E26" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>46078</v>
+      </c>
+      <c r="B27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Teclado Mecânico KeyStorm</v>
+      </c>
+      <c r="D27" s="4">
+        <v>22</v>
+      </c>
+      <c r="E27" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>46079</v>
+      </c>
+      <c r="B28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Webcam Full HD VisionCam</v>
+      </c>
+      <c r="D28" s="4">
+        <v>25</v>
+      </c>
+      <c r="E28" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>46080</v>
+      </c>
+      <c r="B29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Power Bank 10000mAh</v>
+      </c>
+      <c r="D29" s="4">
+        <v>40</v>
+      </c>
+      <c r="E29" t="s">
+        <v>77</v>
+      </c>
+      <c r="F29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Luminária LED Smart</v>
+      </c>
+      <c r="D30" s="4">
+        <v>18</v>
+      </c>
+      <c r="E30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B31" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" t="str">
+        <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
+        <v>Roteador Wi-Fi Dual Band</v>
+      </c>
+      <c r="D31" s="4">
+        <v>26</v>
+      </c>
+      <c r="E31" t="s">
+        <v>79</v>
+      </c>
+      <c r="F31" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F36" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
cria resumo analitico de estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C36FD7-61D8-4E87-B3D6-2253019FCA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C4DCE2-2ECB-4142-BBB2-90E2612CE3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro" sheetId="1" r:id="rId1"/>
     <sheet name="Entrada" sheetId="2" r:id="rId2"/>
     <sheet name="Saída" sheetId="3" r:id="rId3"/>
+    <sheet name="Resumo Estoque" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,8 +41,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="87">
   <si>
     <t>SKU</t>
   </si>
@@ -287,14 +310,30 @@
   </si>
   <si>
     <t>Campanha promocional</t>
+  </si>
+  <si>
+    <t>Total Entradas</t>
+  </si>
+  <si>
+    <t>Total Saídas</t>
+  </si>
+  <si>
+    <t>Saldo Atual</t>
+  </si>
+  <si>
+    <t>Valor em Estoque</t>
+  </si>
+  <si>
+    <t>Status do Produto</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -333,17 +372,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -389,9 +453,9 @@
     <tableColumn id="2" xr3:uid="{474B68BA-BE3F-4822-A13D-98B92741539B}" name="Produto"/>
     <tableColumn id="3" xr3:uid="{C9C1ED03-FCD0-490A-AE7B-3D65AB9EBFBB}" name="Descrição"/>
     <tableColumn id="4" xr3:uid="{8BEC5BD3-48D4-4690-B9D3-B90E65A45828}" name="Categoria"/>
-    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="15"/>
     <tableColumn id="6" xr3:uid="{EA58917D-0C34-4FB2-A614-DCAD68AA44F6}" name="Fornecedor"/>
-    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -401,12 +465,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}" name="tbEntrada" displayName="tbEntrada" ref="A1:F26" totalsRowShown="0">
   <autoFilter ref="A1:F26" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{7987F022-B4FC-4F00-B1FF-6BFCB106433D}" name="SKU"/>
-    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="12">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="11"/>
     <tableColumn id="5" xr3:uid="{575BEAB7-E3EC-442C-9D56-D43256ABCBFE}" name="Responsável"/>
     <tableColumn id="6" xr3:uid="{3F64F76D-003F-4F5F-B825-2C63E0C4FEBC}" name="Observação"/>
   </tableColumns>
@@ -418,12 +482,46 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}" name="tbSaida" displayName="tbSaida" ref="A1:F31" totalsRowShown="0">
   <autoFilter ref="A1:F31" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{84870D34-BE9F-4CFC-A62B-6EE2B5631FD5}" name="Data" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{84870D34-BE9F-4CFC-A62B-6EE2B5631FD5}" name="Data" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{73BFB05B-0638-42FE-83E0-AB0F3445B4FF}" name="SKU"/>
-    <tableColumn id="3" xr3:uid="{63B5D954-F021-49FF-BBD4-26F9DF540E6B}" name="Produto" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{C7872616-E7BA-4C77-8D41-2068067BB2A7}" name="Quantidade Saída" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{63B5D954-F021-49FF-BBD4-26F9DF540E6B}" name="Produto" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{C7872616-E7BA-4C77-8D41-2068067BB2A7}" name="Quantidade Saída" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{9B35AB08-6C54-43E0-B34D-15830AD4E19C}" name="Canal de Venda"/>
     <tableColumn id="6" xr3:uid="{AB3D24CB-C511-41D2-9E6C-DBF4DB411643}" name="Observação"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BD7C1072-069C-4E65-BC46-A0126DC66A9D}" name="tbResumo" displayName="tbResumo" ref="A1:I16" totalsRowShown="0">
+  <autoFilter ref="A1:I16" xr:uid="{BD7C1072-069C-4E65-BC46-A0126DC66A9D}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{AFCC0670-0435-4226-9FA6-3F4C4570978C}" name="SKU"/>
+    <tableColumn id="2" xr3:uid="{33970285-D1D7-476B-BBA9-8275F1325098}" name="Produto" dataDxfId="7">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{FBE19390-9F20-412F-B9BC-5B2C4EDF63CC}" name="Categoria" dataDxfId="6">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{835D2E0F-0263-42D6-AA0A-94AF4AA5E9F9}" name="Preço Unitário" dataDxfId="5">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{942FB79E-E6A3-41AC-9404-32FE05DC1B9B}" name="Total Entradas" dataDxfId="3">
+      <calculatedColumnFormula>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{7BEFCDA8-EFA9-4C2A-8C16-E8BC7BC238F9}" name="Total Saídas" dataDxfId="2">
+      <calculatedColumnFormula>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{5D9EA3A2-6461-4B5F-B087-6EF35C8877D7}" name="Saldo Atual" dataDxfId="0">
+      <calculatedColumnFormula>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{BD3FFB3C-1AD7-4CB3-B102-E85977A14914}" name="Valor em Estoque" dataDxfId="1">
+      <calculatedColumnFormula>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{09CD25CB-684F-43EF-9564-9897A61DFF8E}" name="Status do Produto" dataDxfId="4">
+      <calculatedColumnFormula array="1">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2369,4 +2467,611 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78EF1823-38DC-4F13-BD7D-D83D5208BED0}">
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="18.21875" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Fone Bluetooth AirMax</v>
+      </c>
+      <c r="C2" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Áudio</v>
+      </c>
+      <c r="D2" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>129.9</v>
+      </c>
+      <c r="E2" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>110</v>
+      </c>
+      <c r="F2" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>37</v>
+      </c>
+      <c r="G2" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>73</v>
+      </c>
+      <c r="H2" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>9482.7000000000007</v>
+      </c>
+      <c r="I2" t="str" cm="1">
+        <f t="array" ref="I2">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Caixa de Som MiniBass</v>
+      </c>
+      <c r="C3" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Áudio</v>
+      </c>
+      <c r="D3" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>89.9</v>
+      </c>
+      <c r="E3" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>60</v>
+      </c>
+      <c r="F3" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>26</v>
+      </c>
+      <c r="G3" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>34</v>
+      </c>
+      <c r="H3" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>3056.6000000000004</v>
+      </c>
+      <c r="I3" t="str" cm="1">
+        <f t="array" ref="I3">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Mouse Gamer ProClick</v>
+      </c>
+      <c r="C4" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Periféricos</v>
+      </c>
+      <c r="D4" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>79.900000000000006</v>
+      </c>
+      <c r="E4" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>135</v>
+      </c>
+      <c r="F4" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>52</v>
+      </c>
+      <c r="G4" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>83</v>
+      </c>
+      <c r="H4" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>6631.7000000000007</v>
+      </c>
+      <c r="I4" t="str" cm="1">
+        <f t="array" ref="I4">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Teclado Mecânico KeyStorm</v>
+      </c>
+      <c r="C5" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Periféricos</v>
+      </c>
+      <c r="D5" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>219.9</v>
+      </c>
+      <c r="E5" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>45</v>
+      </c>
+      <c r="F5" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>32</v>
+      </c>
+      <c r="G5" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>13</v>
+      </c>
+      <c r="H5" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>2858.7000000000003</v>
+      </c>
+      <c r="I5" t="str" cm="1">
+        <f t="array" ref="I5">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>Crítico</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Webcam Full HD VisionCam</v>
+      </c>
+      <c r="C6" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Periféricos</v>
+      </c>
+      <c r="D6" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>159.9</v>
+      </c>
+      <c r="E6" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>50</v>
+      </c>
+      <c r="F6" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>40</v>
+      </c>
+      <c r="G6" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>10</v>
+      </c>
+      <c r="H6" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>1599</v>
+      </c>
+      <c r="I6" t="str" cm="1">
+        <f t="array" ref="I6">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>Crítico</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Carregador USB-C Turbo</v>
+      </c>
+      <c r="C7" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Acessórios</v>
+      </c>
+      <c r="D7" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>69.900000000000006</v>
+      </c>
+      <c r="E7" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>170</v>
+      </c>
+      <c r="F7" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>83</v>
+      </c>
+      <c r="G7" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>87</v>
+      </c>
+      <c r="H7" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>6081.3</v>
+      </c>
+      <c r="I7" t="str" cm="1">
+        <f t="array" ref="I7">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Cabo USB-C Reforçado</v>
+      </c>
+      <c r="C8" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Acessórios</v>
+      </c>
+      <c r="D8" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>29.9</v>
+      </c>
+      <c r="E8" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>300</v>
+      </c>
+      <c r="F8" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>165</v>
+      </c>
+      <c r="G8" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>135</v>
+      </c>
+      <c r="H8" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>4036.5</v>
+      </c>
+      <c r="I8" t="str" cm="1">
+        <f t="array" ref="I8">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>Excesso</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Power Bank 10000mAh</v>
+      </c>
+      <c r="C9" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Acessórios</v>
+      </c>
+      <c r="D9" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>119.9</v>
+      </c>
+      <c r="E9" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>90</v>
+      </c>
+      <c r="F9" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>58</v>
+      </c>
+      <c r="G9" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>32</v>
+      </c>
+      <c r="H9" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>3836.8</v>
+      </c>
+      <c r="I9" t="str" cm="1">
+        <f t="array" ref="I9">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Luminária LED Smart</v>
+      </c>
+      <c r="C10" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Casa Inteligente</v>
+      </c>
+      <c r="D10" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>149.9</v>
+      </c>
+      <c r="E10" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>40</v>
+      </c>
+      <c r="F10" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>27</v>
+      </c>
+      <c r="G10" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>13</v>
+      </c>
+      <c r="H10" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>1948.7</v>
+      </c>
+      <c r="I10" t="str" cm="1">
+        <f t="array" ref="I10">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>Crítico</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Tomada Inteligente Wi-Fi</v>
+      </c>
+      <c r="C11" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Casa Inteligente</v>
+      </c>
+      <c r="D11" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>99.9</v>
+      </c>
+      <c r="E11" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>90</v>
+      </c>
+      <c r="F11" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>36</v>
+      </c>
+      <c r="G11" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>54</v>
+      </c>
+      <c r="H11" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>5394.6</v>
+      </c>
+      <c r="I11" t="str" cm="1">
+        <f t="array" ref="I11">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Roteador Wi-Fi Dual Band</v>
+      </c>
+      <c r="C12" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Redes</v>
+      </c>
+      <c r="D12" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>189.9</v>
+      </c>
+      <c r="E12" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>55</v>
+      </c>
+      <c r="F12" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>40</v>
+      </c>
+      <c r="G12" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>15</v>
+      </c>
+      <c r="H12" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>2848.5</v>
+      </c>
+      <c r="I12" t="str" cm="1">
+        <f t="array" ref="I12">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>Crítico</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Repetidor de Sinal Wi-Fi</v>
+      </c>
+      <c r="C13" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Redes</v>
+      </c>
+      <c r="D13" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>109.9</v>
+      </c>
+      <c r="E13" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>105</v>
+      </c>
+      <c r="F13" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>57</v>
+      </c>
+      <c r="G13" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>48</v>
+      </c>
+      <c r="H13" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>5275.2000000000007</v>
+      </c>
+      <c r="I13" t="str" cm="1">
+        <f t="array" ref="I13">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>SSD 480GB FastDisk</v>
+      </c>
+      <c r="C14" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Armazenamento</v>
+      </c>
+      <c r="D14" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>259.89999999999998</v>
+      </c>
+      <c r="E14" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>130</v>
+      </c>
+      <c r="F14" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>72</v>
+      </c>
+      <c r="G14" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>58</v>
+      </c>
+      <c r="H14" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>15074.199999999999</v>
+      </c>
+      <c r="I14" t="str" cm="1">
+        <f t="array" ref="I14">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Pendrive 64GB DataGo</v>
+      </c>
+      <c r="C15" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Armazenamento</v>
+      </c>
+      <c r="D15" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>49.9</v>
+      </c>
+      <c r="E15" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>230</v>
+      </c>
+      <c r="F15" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>170</v>
+      </c>
+      <c r="G15" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>60</v>
+      </c>
+      <c r="H15" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>2994</v>
+      </c>
+      <c r="I15" t="str" cm="1">
+        <f t="array" ref="I15">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
+        <v>Hub USB 4 Portas</v>
+      </c>
+      <c r="C16" t="str">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
+        <v>Acessórios</v>
+      </c>
+      <c r="D16" s="5">
+        <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
+        <v>59.9</v>
+      </c>
+      <c r="E16" s="4">
+        <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>155</v>
+      </c>
+      <c r="F16" s="4">
+        <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
+        <v>78</v>
+      </c>
+      <c r="G16" s="4">
+        <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
+        <v>77</v>
+      </c>
+      <c r="H16" s="5">
+        <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
+        <v>4612.3</v>
+      </c>
+      <c r="I16" t="str" cm="1">
+        <f t="array" ref="I16">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</f>
+        <v>OK</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
aplica formatacao condicional no resumo de estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C4DCE2-2ECB-4142-BBB2-90E2612CE3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7543E0-04AA-47F7-B82A-46BCCC185628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
@@ -383,7 +383,594 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="81">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -453,9 +1040,9 @@
     <tableColumn id="2" xr3:uid="{474B68BA-BE3F-4822-A13D-98B92741539B}" name="Produto"/>
     <tableColumn id="3" xr3:uid="{C9C1ED03-FCD0-490A-AE7B-3D65AB9EBFBB}" name="Descrição"/>
     <tableColumn id="4" xr3:uid="{8BEC5BD3-48D4-4690-B9D3-B90E65A45828}" name="Categoria"/>
-    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{436AE5E3-8707-4267-BC04-5D2C9A67A0FC}" name="Preço Unitário" dataDxfId="80"/>
     <tableColumn id="6" xr3:uid="{EA58917D-0C34-4FB2-A614-DCAD68AA44F6}" name="Fornecedor"/>
-    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{04EAC182-50EF-47E6-BCFB-5A3CF1673859}" name="Data de Cadastro" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -465,12 +1052,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}" name="tbEntrada" displayName="tbEntrada" ref="A1:F26" totalsRowShown="0">
   <autoFilter ref="A1:F26" xr:uid="{E47F13DD-B86B-492C-98DA-F2F5B2C8D8F6}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E9596E97-1BC4-4840-8827-C2762EA08DF0}" name="Data" dataDxfId="78"/>
     <tableColumn id="2" xr3:uid="{7987F022-B4FC-4F00-B1FF-6BFCB106433D}" name="SKU"/>
-    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{CE0AFAD0-D886-4AD3-9DC7-F53B9E49B62D}" name="Produto" dataDxfId="77">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{1B8D7365-FCDC-4BA4-8560-936671FD7ACB}" name="Quantidade Entrada" dataDxfId="76"/>
     <tableColumn id="5" xr3:uid="{575BEAB7-E3EC-442C-9D56-D43256ABCBFE}" name="Responsável"/>
     <tableColumn id="6" xr3:uid="{3F64F76D-003F-4F5F-B825-2C63E0C4FEBC}" name="Observação"/>
   </tableColumns>
@@ -482,10 +1069,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}" name="tbSaida" displayName="tbSaida" ref="A1:F31" totalsRowShown="0">
   <autoFilter ref="A1:F31" xr:uid="{83603194-BD4A-445E-92EE-AEDDA93B7FEE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{84870D34-BE9F-4CFC-A62B-6EE2B5631FD5}" name="Data" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{84870D34-BE9F-4CFC-A62B-6EE2B5631FD5}" name="Data" dataDxfId="75"/>
     <tableColumn id="2" xr3:uid="{73BFB05B-0638-42FE-83E0-AB0F3445B4FF}" name="SKU"/>
-    <tableColumn id="3" xr3:uid="{63B5D954-F021-49FF-BBD4-26F9DF540E6B}" name="Produto" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{C7872616-E7BA-4C77-8D41-2068067BB2A7}" name="Quantidade Saída" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{63B5D954-F021-49FF-BBD4-26F9DF540E6B}" name="Produto" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{C7872616-E7BA-4C77-8D41-2068067BB2A7}" name="Quantidade Saída" dataDxfId="73"/>
     <tableColumn id="5" xr3:uid="{9B35AB08-6C54-43E0-B34D-15830AD4E19C}" name="Canal de Venda"/>
     <tableColumn id="6" xr3:uid="{AB3D24CB-C511-41D2-9E6C-DBF4DB411643}" name="Observação"/>
   </tableColumns>
@@ -498,28 +1085,28 @@
   <autoFilter ref="A1:I16" xr:uid="{BD7C1072-069C-4E65-BC46-A0126DC66A9D}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{AFCC0670-0435-4226-9FA6-3F4C4570978C}" name="SKU"/>
-    <tableColumn id="2" xr3:uid="{33970285-D1D7-476B-BBA9-8275F1325098}" name="Produto" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{33970285-D1D7-476B-BBA9-8275F1325098}" name="Produto" dataDxfId="72">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{FBE19390-9F20-412F-B9BC-5B2C4EDF63CC}" name="Categoria" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{FBE19390-9F20-412F-B9BC-5B2C4EDF63CC}" name="Categoria" dataDxfId="71">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{835D2E0F-0263-42D6-AA0A-94AF4AA5E9F9}" name="Preço Unitário" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{835D2E0F-0263-42D6-AA0A-94AF4AA5E9F9}" name="Preço Unitário" dataDxfId="70">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{942FB79E-E6A3-41AC-9404-32FE05DC1B9B}" name="Total Entradas" dataDxfId="3">
+    <tableColumn id="5" xr3:uid="{942FB79E-E6A3-41AC-9404-32FE05DC1B9B}" name="Total Entradas" dataDxfId="68">
       <calculatedColumnFormula>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{7BEFCDA8-EFA9-4C2A-8C16-E8BC7BC238F9}" name="Total Saídas" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{7BEFCDA8-EFA9-4C2A-8C16-E8BC7BC238F9}" name="Total Saídas" dataDxfId="67">
       <calculatedColumnFormula>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5D9EA3A2-6461-4B5F-B087-6EF35C8877D7}" name="Saldo Atual" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{5D9EA3A2-6461-4B5F-B087-6EF35C8877D7}" name="Saldo Atual" dataDxfId="65">
       <calculatedColumnFormula>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BD3FFB3C-1AD7-4CB3-B102-E85977A14914}" name="Valor em Estoque" dataDxfId="1">
+    <tableColumn id="8" xr3:uid="{BD3FFB3C-1AD7-4CB3-B102-E85977A14914}" name="Valor em Estoque" dataDxfId="66">
       <calculatedColumnFormula>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{09CD25CB-684F-43EF-9564-9897A61DFF8E}" name="Status do Produto" dataDxfId="4">
+    <tableColumn id="9" xr3:uid="{09CD25CB-684F-43EF-9564-9897A61DFF8E}" name="Status do Produto" dataDxfId="69">
       <calculatedColumnFormula array="1">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2480,7 +3067,7 @@
     <col min="5" max="5" width="15.33203125" style="4" customWidth="1"/>
     <col min="6" max="6" width="16.21875" style="4" customWidth="1"/>
     <col min="7" max="7" width="15.21875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="18.21875" customWidth="1"/>
+    <col min="8" max="8" width="25.109375" customWidth="1"/>
     <col min="9" max="9" width="18.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3035,7 +3622,7 @@
       <c r="A16" t="s">
         <v>63</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B16" s="3" t="str">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"Não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
@@ -3069,9 +3656,76 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="I2:I1048576">
+    <cfRule type="containsText" dxfId="19" priority="11" operator="containsText" text="Estoque Negativo">
+      <formula>NOT(ISERROR(SEARCH("Estoque Negativo",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="10" operator="containsText" text="Obsoleto">
+      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="9" operator="containsText" text="Obsoleto">
+      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="8" operator="containsText" text="Crítico">
+      <formula>NOT(ISERROR(SEARCH("Crítico",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="OK">
+      <formula>NOT(ISERROR(SEARCH("OK",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="Excesso">
+      <formula>NOT(ISERROR(SEARCH("Excesso",I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G1048576">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="between">
+      <formula>1</formula>
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="greaterThan">
+      <formula>100</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="between">
+      <formula>21</formula>
+      <formula>99</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H1048576">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{C20CB109-B948-4D59-A50C-2622DC3F61EC}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{C20CB109-B948-4D59-A50C-2622DC3F61EC}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H2:H1048576</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cria tabelas dinamicas de estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -8,17 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7543E0-04AA-47F7-B82A-46BCCC185628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD9141AB-DDA8-4E5D-8E95-9710A94CAD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro" sheetId="1" r:id="rId1"/>
     <sheet name="Entrada" sheetId="2" r:id="rId2"/>
     <sheet name="Saída" sheetId="3" r:id="rId3"/>
     <sheet name="Resumo Estoque" sheetId="4" r:id="rId4"/>
+    <sheet name="Tabelas Dinâmicas" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="11" r:id="rId6"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -64,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="102">
   <si>
     <t>SKU</t>
   </si>
@@ -325,6 +329,51 @@
   </si>
   <si>
     <t>Status do Produto</t>
+  </si>
+  <si>
+    <t>Rótulos de Linha</t>
+  </si>
+  <si>
+    <t>Total Geral</t>
+  </si>
+  <si>
+    <t>Soma de Valor em Estoque</t>
+  </si>
+  <si>
+    <t>Valor total em estoque por categoria</t>
+  </si>
+  <si>
+    <t>Contagem de SKU</t>
+  </si>
+  <si>
+    <t>Quantidade de SKUs por categoria</t>
+  </si>
+  <si>
+    <t>Média de Preço Unitário</t>
+  </si>
+  <si>
+    <t>Preço médio por categoria</t>
+  </si>
+  <si>
+    <t>Soma de Total Entradas</t>
+  </si>
+  <si>
+    <t>Total de saídas por categoria</t>
+  </si>
+  <si>
+    <t>Crítico</t>
+  </si>
+  <si>
+    <t>Excesso</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Produtos por status</t>
+  </si>
+  <si>
+    <t>Top produtos por valor em estoque</t>
   </si>
 </sst>
 </file>
@@ -372,13 +421,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1030,6 +1084,740 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jarleson Oliveira" refreshedDate="46148.552556249997" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="15" xr:uid="{9BEAD0A7-2E1C-46B7-9BF7-BD42310BF8B2}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="tbResumo"/>
+  </cacheSource>
+  <cacheFields count="9">
+    <cacheField name="SKU" numFmtId="0">
+      <sharedItems count="15">
+        <s v="SKU001"/>
+        <s v="SKU002"/>
+        <s v="SKU003"/>
+        <s v="SKU004"/>
+        <s v="SKU005"/>
+        <s v="SKU006"/>
+        <s v="SKU007"/>
+        <s v="SKU008"/>
+        <s v="SKU009"/>
+        <s v="SKU010"/>
+        <s v="SKU011"/>
+        <s v="SKU012"/>
+        <s v="SKU013"/>
+        <s v="SKU014"/>
+        <s v="SKU015"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Produto" numFmtId="0">
+      <sharedItems count="15">
+        <s v="Fone Bluetooth AirMax"/>
+        <s v="Caixa de Som MiniBass"/>
+        <s v="Mouse Gamer ProClick"/>
+        <s v="Teclado Mecânico KeyStorm"/>
+        <s v="Webcam Full HD VisionCam"/>
+        <s v="Carregador USB-C Turbo"/>
+        <s v="Cabo USB-C Reforçado"/>
+        <s v="Power Bank 10000mAh"/>
+        <s v="Luminária LED Smart"/>
+        <s v="Tomada Inteligente Wi-Fi"/>
+        <s v="Roteador Wi-Fi Dual Band"/>
+        <s v="Repetidor de Sinal Wi-Fi"/>
+        <s v="SSD 480GB FastDisk"/>
+        <s v="Pendrive 64GB DataGo"/>
+        <s v="Hub USB 4 Portas"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Categoria" numFmtId="0">
+      <sharedItems count="6">
+        <s v="Áudio"/>
+        <s v="Periféricos"/>
+        <s v="Acessórios"/>
+        <s v="Casa Inteligente"/>
+        <s v="Redes"/>
+        <s v="Armazenamento"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Preço Unitário" numFmtId="168">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="29.9" maxValue="259.89999999999998"/>
+    </cacheField>
+    <cacheField name="Total Entradas" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="40" maxValue="300"/>
+    </cacheField>
+    <cacheField name="Total Saídas" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="26" maxValue="170"/>
+    </cacheField>
+    <cacheField name="Saldo Atual" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="10" maxValue="135"/>
+    </cacheField>
+    <cacheField name="Valor em Estoque" numFmtId="168">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1599" maxValue="15074.199999999999"/>
+    </cacheField>
+    <cacheField name="Status do Produto" numFmtId="0">
+      <sharedItems count="3">
+        <s v="OK"/>
+        <s v="Crítico"/>
+        <s v="Excesso"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="15">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="129.9"/>
+    <n v="110"/>
+    <n v="37"/>
+    <n v="73"/>
+    <n v="9482.7000000000007"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="89.9"/>
+    <n v="60"/>
+    <n v="26"/>
+    <n v="34"/>
+    <n v="3056.6000000000004"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="79.900000000000006"/>
+    <n v="135"/>
+    <n v="52"/>
+    <n v="83"/>
+    <n v="6631.7000000000007"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="219.9"/>
+    <n v="45"/>
+    <n v="32"/>
+    <n v="13"/>
+    <n v="2858.7000000000003"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="159.9"/>
+    <n v="50"/>
+    <n v="40"/>
+    <n v="10"/>
+    <n v="1599"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="5"/>
+    <x v="2"/>
+    <n v="69.900000000000006"/>
+    <n v="170"/>
+    <n v="83"/>
+    <n v="87"/>
+    <n v="6081.3"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="29.9"/>
+    <n v="300"/>
+    <n v="165"/>
+    <n v="135"/>
+    <n v="4036.5"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="7"/>
+    <x v="2"/>
+    <n v="119.9"/>
+    <n v="90"/>
+    <n v="58"/>
+    <n v="32"/>
+    <n v="3836.8"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="8"/>
+    <x v="3"/>
+    <n v="149.9"/>
+    <n v="40"/>
+    <n v="27"/>
+    <n v="13"/>
+    <n v="1948.7"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="9"/>
+    <x v="3"/>
+    <n v="99.9"/>
+    <n v="90"/>
+    <n v="36"/>
+    <n v="54"/>
+    <n v="5394.6"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="10"/>
+    <x v="10"/>
+    <x v="4"/>
+    <n v="189.9"/>
+    <n v="55"/>
+    <n v="40"/>
+    <n v="15"/>
+    <n v="2848.5"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="11"/>
+    <x v="11"/>
+    <x v="4"/>
+    <n v="109.9"/>
+    <n v="105"/>
+    <n v="57"/>
+    <n v="48"/>
+    <n v="5275.2000000000007"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="12"/>
+    <x v="12"/>
+    <x v="5"/>
+    <n v="259.89999999999998"/>
+    <n v="130"/>
+    <n v="72"/>
+    <n v="58"/>
+    <n v="15074.199999999999"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="13"/>
+    <x v="13"/>
+    <x v="5"/>
+    <n v="49.9"/>
+    <n v="230"/>
+    <n v="170"/>
+    <n v="60"/>
+    <n v="2994"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="14"/>
+    <x v="14"/>
+    <x v="2"/>
+    <n v="59.9"/>
+    <n v="155"/>
+    <n v="78"/>
+    <n v="77"/>
+    <n v="4612.3"/>
+    <x v="0"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9AD11E86-4924-4261-BC83-101B6E91C0CF}" name="Tabela dinâmica6" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="D15:E31" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="16">
+        <item x="6"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="14"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="168" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="16">
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma de Valor em Estoque" fld="7" baseField="0" baseItem="0" numFmtId="168"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5AB161A-AD5E-4FF1-AE61-3A2B15A1C384}" name="Tabela dinâmica5" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A15:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField dataField="1" showAll="0">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de SKU" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4D1C298E-F488-450E-81B0-61195D914338}" name="Tabela dinâmica4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="J3:K10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField dataField="1" numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma de Total Entradas" fld="4" baseField="0" baseItem="0" numFmtId="1"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5282D270-EAFA-470E-9420-AE022D18FC38}" name="Tabela dinâmica3" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="G3:H10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Média de Preço Unitário" fld="3" subtotal="average" baseField="2" baseItem="0" numFmtId="168"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FFAF811-45F8-4D93-8D26-D6178C957874}" name="Tabela dinâmica2" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="D3:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField dataField="1" showAll="0">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de SKU" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FCE78C11-AF54-4448-B789-406373CF54CE}" name="Tabela dinâmica1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="168" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma de Valor em Estoque" fld="7" baseField="2" baseItem="0" numFmtId="168"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1830,7 +2618,7 @@
     <col min="1" max="1" width="15.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" customWidth="1"/>
     <col min="3" max="3" width="28.88671875" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="5" customWidth="1"/>
     <col min="5" max="5" width="21.44140625" customWidth="1"/>
     <col min="6" max="6" width="26.109375" customWidth="1"/>
   </cols>
@@ -1845,7 +2633,7 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E1" t="s">
@@ -1866,7 +2654,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
         <v>80</v>
       </c>
       <c r="E2" t="s">
@@ -1887,7 +2675,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Caixa de Som MiniBass</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="5">
         <v>60</v>
       </c>
       <c r="E3" t="s">
@@ -1908,7 +2696,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>100</v>
       </c>
       <c r="E4" t="s">
@@ -1929,7 +2717,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Teclado Mecânico KeyStorm</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>45</v>
       </c>
       <c r="E5" t="s">
@@ -1950,7 +2738,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Webcam Full HD VisionCam</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>50</v>
       </c>
       <c r="E6" t="s">
@@ -1971,7 +2759,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>120</v>
       </c>
       <c r="E7" t="s">
@@ -1992,7 +2780,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>200</v>
       </c>
       <c r="E8" t="s">
@@ -2013,7 +2801,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>70</v>
       </c>
       <c r="E9" t="s">
@@ -2034,7 +2822,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <v>40</v>
       </c>
       <c r="E10" t="s">
@@ -2055,7 +2843,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="5">
         <v>65</v>
       </c>
       <c r="E11" t="s">
@@ -2076,7 +2864,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="5">
         <v>55</v>
       </c>
       <c r="E12" t="s">
@@ -2097,7 +2885,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="5">
         <v>75</v>
       </c>
       <c r="E13" t="s">
@@ -2118,7 +2906,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="5">
         <v>90</v>
       </c>
       <c r="E14" t="s">
@@ -2139,7 +2927,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="5">
         <v>150</v>
       </c>
       <c r="E15" t="s">
@@ -2160,7 +2948,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="5">
         <v>110</v>
       </c>
       <c r="E16" t="s">
@@ -2181,7 +2969,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="5">
         <v>30</v>
       </c>
       <c r="E17" t="s">
@@ -2202,7 +2990,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="5">
         <v>50</v>
       </c>
       <c r="E18" t="s">
@@ -2223,7 +3011,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="5">
         <v>100</v>
       </c>
       <c r="E19" t="s">
@@ -2244,7 +3032,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="5">
         <v>40</v>
       </c>
       <c r="E20" t="s">
@@ -2265,7 +3053,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="5">
         <v>80</v>
       </c>
       <c r="E21" t="s">
@@ -2286,7 +3074,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="5">
         <v>35</v>
       </c>
       <c r="E22" t="s">
@@ -2307,7 +3095,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="5">
         <v>25</v>
       </c>
       <c r="E23" t="s">
@@ -2328,7 +3116,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="5">
         <v>30</v>
       </c>
       <c r="E24" t="s">
@@ -2349,7 +3137,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="5">
         <v>45</v>
       </c>
       <c r="E25" t="s">
@@ -2370,7 +3158,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="5">
         <v>20</v>
       </c>
       <c r="E26" t="s">
@@ -2396,7 +3184,7 @@
     <col min="1" max="1" width="16.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" customWidth="1"/>
     <col min="3" max="3" width="20.5546875" customWidth="1"/>
-    <col min="4" max="4" width="26.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="26.44140625" style="5" customWidth="1"/>
     <col min="5" max="5" width="24.21875" customWidth="1"/>
     <col min="6" max="6" width="26.44140625" customWidth="1"/>
   </cols>
@@ -2411,7 +3199,7 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>75</v>
       </c>
       <c r="E1" t="s">
@@ -2431,7 +3219,7 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
         <v>12</v>
       </c>
       <c r="E2" t="s">
@@ -2451,7 +3239,7 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="5">
         <v>8</v>
       </c>
       <c r="E3" t="s">
@@ -2471,7 +3259,7 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>20</v>
       </c>
       <c r="E4" t="s">
@@ -2491,7 +3279,7 @@
       <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>10</v>
       </c>
       <c r="E5" t="s">
@@ -2511,7 +3299,7 @@
       <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>15</v>
       </c>
       <c r="E6" t="s">
@@ -2531,7 +3319,7 @@
       <c r="C7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>35</v>
       </c>
       <c r="E7" t="s">
@@ -2552,7 +3340,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>70</v>
       </c>
       <c r="E8" t="s">
@@ -2573,7 +3361,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>18</v>
       </c>
       <c r="E9" t="s">
@@ -2594,7 +3382,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <v>9</v>
       </c>
       <c r="E10" t="s">
@@ -2615,7 +3403,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="5">
         <v>16</v>
       </c>
       <c r="E11" t="s">
@@ -2636,7 +3424,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="5">
         <v>14</v>
       </c>
       <c r="E12" t="s">
@@ -2657,7 +3445,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="5">
         <v>22</v>
       </c>
       <c r="E13" t="s">
@@ -2678,7 +3466,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="5">
         <v>30</v>
       </c>
       <c r="E14" t="s">
@@ -2699,7 +3487,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="5">
         <v>60</v>
       </c>
       <c r="E15" t="s">
@@ -2720,7 +3508,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="5">
         <v>28</v>
       </c>
       <c r="E16" t="s">
@@ -2741,7 +3529,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="5">
         <v>25</v>
       </c>
       <c r="E17" t="s">
@@ -2762,7 +3550,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="5">
         <v>32</v>
       </c>
       <c r="E18" t="s">
@@ -2783,7 +3571,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="5">
         <v>48</v>
       </c>
       <c r="E19" t="s">
@@ -2804,7 +3592,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="5">
         <v>95</v>
       </c>
       <c r="E20" t="s">
@@ -2825,7 +3613,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="5">
         <v>42</v>
       </c>
       <c r="E21" t="s">
@@ -2846,7 +3634,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="5">
         <v>110</v>
       </c>
       <c r="E22" t="s">
@@ -2867,7 +3655,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="5">
         <v>20</v>
       </c>
       <c r="E23" t="s">
@@ -2888,7 +3676,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="5">
         <v>35</v>
       </c>
       <c r="E24" t="s">
@@ -2909,7 +3697,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="5">
         <v>50</v>
       </c>
       <c r="E25" t="s">
@@ -2930,7 +3718,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Caixa de Som MiniBass</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="5">
         <v>18</v>
       </c>
       <c r="E26" t="s">
@@ -2951,7 +3739,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Teclado Mecânico KeyStorm</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="5">
         <v>22</v>
       </c>
       <c r="E27" t="s">
@@ -2972,7 +3760,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Webcam Full HD VisionCam</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="5">
         <v>25</v>
       </c>
       <c r="E28" t="s">
@@ -2993,7 +3781,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="5">
         <v>40</v>
       </c>
       <c r="E29" t="s">
@@ -3014,7 +3802,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D30" s="4">
+      <c r="D30" s="5">
         <v>18</v>
       </c>
       <c r="E30" t="s">
@@ -3035,7 +3823,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D31" s="5">
         <v>26</v>
       </c>
       <c r="E31" t="s">
@@ -3063,10 +3851,10 @@
   <cols>
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
     <col min="3" max="3" width="26.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" style="5" customWidth="1"/>
     <col min="8" max="8" width="25.109375" customWidth="1"/>
     <col min="9" max="9" width="18.44140625" customWidth="1"/>
   </cols>
@@ -3081,16 +3869,16 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>84</v>
       </c>
       <c r="H1" t="s">
@@ -3112,23 +3900,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Áudio</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>129.9</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>110</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>37</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>73</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>9482.7000000000007</v>
       </c>
@@ -3149,23 +3937,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Áudio</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>89.9</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>60</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>26</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>34</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>3056.6000000000004</v>
       </c>
@@ -3186,23 +3974,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>79.900000000000006</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>135</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>52</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>83</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>6631.7000000000007</v>
       </c>
@@ -3223,23 +4011,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>219.9</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>45</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>32</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>13</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2858.7000000000003</v>
       </c>
@@ -3260,23 +4048,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>159.9</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>50</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>10</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>1599</v>
       </c>
@@ -3297,23 +4085,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>69.900000000000006</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>170</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>83</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>87</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>6081.3</v>
       </c>
@@ -3334,23 +4122,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>29.9</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>300</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>165</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>135</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>4036.5</v>
       </c>
@@ -3371,23 +4159,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>119.9</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>90</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>58</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>32</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>3836.8</v>
       </c>
@@ -3408,23 +4196,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Casa Inteligente</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>149.9</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>27</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>13</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>1948.7</v>
       </c>
@@ -3445,23 +4233,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Casa Inteligente</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>99.9</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>90</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>36</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>54</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>5394.6</v>
       </c>
@@ -3482,23 +4270,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Redes</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>189.9</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>55</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>15</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2848.5</v>
       </c>
@@ -3519,23 +4307,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Redes</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>109.9</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>105</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>57</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>48</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>5275.2000000000007</v>
       </c>
@@ -3556,23 +4344,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Armazenamento</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>259.89999999999998</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>130</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>72</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>58</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>15074.199999999999</v>
       </c>
@@ -3593,23 +4381,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Armazenamento</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>49.9</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>230</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>170</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>60</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2994</v>
       </c>
@@ -3630,23 +4418,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="6">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>59.9</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="5">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>155</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="5">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>78</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="5">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>77</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="6">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>4612.3</v>
       </c>
@@ -3728,4 +4516,420 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DEA12BB-F18F-4295-B22F-A8EBCBD3AB47}">
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.77734375" customWidth="1"/>
+    <col min="11" max="11" width="21.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="6">
+        <v>18566.899999999998</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="4">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="6">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="5">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="6">
+        <v>18068.199999999997</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="4">
+        <v>2</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="6">
+        <v>154.89999999999998</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" s="5">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="6">
+        <v>12539.300000000001</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4">
+        <v>2</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="6">
+        <v>109.9</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="5">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="6">
+        <v>7343.3</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="4">
+        <v>2</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="6">
+        <v>124.9</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" s="5">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="6">
+        <v>11089.400000000001</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4">
+        <v>3</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="6">
+        <v>153.23333333333335</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="5">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="6">
+        <v>8123.7000000000007</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4">
+        <v>2</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="6">
+        <v>149.9</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" s="5">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="6">
+        <v>75730.8</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="4">
+        <v>15</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H10" s="6">
+        <v>121.23333333333336</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="K10" s="5">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="4">
+        <v>4</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="6">
+        <v>15074.199999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="6">
+        <v>9482.7000000000007</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B18" s="4">
+        <v>10</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="6">
+        <v>6631.7000000000007</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="4">
+        <v>15</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="6">
+        <v>6081.3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="6">
+        <v>5394.6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D21" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="6">
+        <v>5275.2000000000007</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D22" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" s="6">
+        <v>4612.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D23" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="6">
+        <v>4036.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D24" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="6">
+        <v>3836.8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="6">
+        <v>3056.6000000000004</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D26" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="6">
+        <v>2994</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D27" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" s="6">
+        <v>2858.7000000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D28" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="6">
+        <v>2848.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D29" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29" s="6">
+        <v>1948.7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D30" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="6">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D31" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" s="6">
+        <v>75730.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
organiza layout do dashboard de estoque
</commit_message>
<xml_diff>
--- a/01-excel-controle-estoque/dashboard-estoque.xlsx
+++ b/01-excel-controle-estoque/dashboard-estoque.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarle\Desktop\Documentosportfolio-data-science\01-excel-controle-estoque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{405524F3-C3A5-4833-ACC7-60ADA6CD2C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480803AE-0BE2-4799-ACF4-0C5DB3BF02B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{9DEF0419-6759-4113-AF76-8A8C57CBF3AA}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="107">
   <si>
     <t>SKU</t>
   </si>
@@ -376,6 +376,21 @@
   <si>
     <t>Top produtos por valor em estoque</t>
   </si>
+  <si>
+    <t>Dashboard de Controle de Estoque — LLC Electronics</t>
+  </si>
+  <si>
+    <t>Valor Total em Estoque</t>
+  </si>
+  <si>
+    <t>Total de SKUs</t>
+  </si>
+  <si>
+    <t>Produtos Críticos</t>
+  </si>
+  <si>
+    <t>Produtos em Excesso</t>
+  </si>
 </sst>
 </file>
 
@@ -383,9 +398,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -401,16 +416,76 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.24994659260841701"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -418,95 +493,118 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyFont="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="60% - Ênfase4" xfId="3" builtinId="44"/>
+    <cellStyle name="Ênfase1" xfId="1" builtinId="29"/>
+    <cellStyle name="Estilo 1" xfId="2" xr:uid="{51C88D06-305F-437F-B5F6-E6E79816B032}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="26">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -528,10 +626,78 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -540,10 +706,10 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -7241,14 +7407,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7278,14 +7444,14 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:colOff>320040</xdr:colOff>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -7317,14 +7483,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7354,15 +7520,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7392,15 +7558,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7430,15 +7596,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>396240</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7522,7 +7688,7 @@
         <s v="Armazenamento"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Preço Unitário" numFmtId="168">
+    <cacheField name="Preço Unitário" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="29.9" maxValue="259.89999999999998"/>
     </cacheField>
     <cacheField name="Total Entradas" numFmtId="1">
@@ -7534,7 +7700,7 @@
     <cacheField name="Saldo Atual" numFmtId="1">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="10" maxValue="135"/>
     </cacheField>
-    <cacheField name="Valor em Estoque" numFmtId="168">
+    <cacheField name="Valor em Estoque" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1599" maxValue="15074.199999999999"/>
     </cacheField>
     <cacheField name="Status do Produto" numFmtId="0">
@@ -7724,7 +7890,184 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9AD11E86-4924-4261-BC83-101B6E91C0CF}" name="Tabela dinâmica6" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FFAF811-45F8-4D93-8D26-D6178C957874}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="D3:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField dataField="1" showAll="0">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de SKU" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FCE78C11-AF54-4448-B789-406373CF54CE}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+  <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma de Valor em Estoque" fld="7" baseField="2" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9AD11E86-4924-4261-BC83-101B6E91C0CF}" name="Tabela dinâmica6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="D15:E31" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -7758,11 +8101,11 @@
       </autoSortScope>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
-    <pivotField dataField="1" numFmtId="168" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -7822,27 +8165,9 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Soma de Valor em Estoque" fld="7" baseField="0" baseItem="0" numFmtId="168"/>
+    <dataField name="Soma de Valor em Estoque" fld="7" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <chartFormats count="3">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="1" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="1">
     <chartFormat chart="2" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -7865,8 +8190,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5AB161A-AD5E-4FF1-AE61-3A2B15A1C384}" name="Tabela dinâmica5" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5AB161A-AD5E-4FF1-AE61-3A2B15A1C384}" name="Tabela dinâmica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A15:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0">
@@ -7891,11 +8216,11 @@
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="4">
         <item x="1"/>
@@ -7928,16 +8253,7 @@
   <dataFields count="1">
     <dataField name="Contagem de SKU" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="5">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="4">
     <chartFormat chart="2" format="5" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -7996,8 +8312,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4D1C298E-F488-450E-81B0-61195D914338}" name="Tabela dinâmica4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4D1C298E-F488-450E-81B0-61195D914338}" name="Tabela dinâmica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="J3:K10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -8013,11 +8329,11 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField dataField="1" numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -8052,16 +8368,7 @@
   <dataFields count="1">
     <dataField name="Soma de Total Entradas" fld="4" baseField="0" baseItem="0" numFmtId="1"/>
   </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="1">
     <chartFormat chart="2" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -8084,8 +8391,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5282D270-EAFA-470E-9420-AE022D18FC38}" name="Tabela dinâmica3" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5282D270-EAFA-470E-9420-AE022D18FC38}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="G3:H10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -8101,11 +8408,11 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField dataField="1" numFmtId="168" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -8138,214 +8445,10 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Média de Preço Unitário" fld="3" subtotal="average" baseField="2" baseItem="0" numFmtId="168"/>
+    <dataField name="Média de Preço Unitário" fld="3" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
+  <chartFormats count="1">
     <chartFormat chart="2" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9FFAF811-45F8-4D93-8D26-D6178C957874}" name="Tabela dinâmica2" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="D3:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField dataField="1" showAll="0">
-      <items count="16">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="168" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="168" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de SKU" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FCE78C11-AF54-4448-B789-406373CF54CE}" name="Tabela dinâmica1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="168" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField dataField="1" numFmtId="168" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma de Valor em Estoque" fld="7" baseField="2" baseItem="0" numFmtId="168"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="2" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -8429,19 +8532,19 @@
     <tableColumn id="4" xr3:uid="{835D2E0F-0263-42D6-AA0A-94AF4AA5E9F9}" name="Preço Unitário" dataDxfId="15">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{942FB79E-E6A3-41AC-9404-32FE05DC1B9B}" name="Total Entradas" dataDxfId="13">
+    <tableColumn id="5" xr3:uid="{942FB79E-E6A3-41AC-9404-32FE05DC1B9B}" name="Total Entradas" dataDxfId="14">
       <calculatedColumnFormula>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{7BEFCDA8-EFA9-4C2A-8C16-E8BC7BC238F9}" name="Total Saídas" dataDxfId="12">
+    <tableColumn id="6" xr3:uid="{7BEFCDA8-EFA9-4C2A-8C16-E8BC7BC238F9}" name="Total Saídas" dataDxfId="13">
       <calculatedColumnFormula>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5D9EA3A2-6461-4B5F-B087-6EF35C8877D7}" name="Saldo Atual" dataDxfId="10">
+    <tableColumn id="7" xr3:uid="{5D9EA3A2-6461-4B5F-B087-6EF35C8877D7}" name="Saldo Atual" dataDxfId="12">
       <calculatedColumnFormula>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{BD3FFB3C-1AD7-4CB3-B102-E85977A14914}" name="Valor em Estoque" dataDxfId="11">
       <calculatedColumnFormula>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{09CD25CB-684F-43EF-9564-9897A61DFF8E}" name="Status do Produto" dataDxfId="14">
+    <tableColumn id="9" xr3:uid="{09CD25CB-684F-43EF-9564-9897A61DFF8E}" name="Status do Produto" dataDxfId="10">
       <calculatedColumnFormula array="1">_xlfn.IFS(tbResumo[[#This Row],[Saldo Atual]]&lt;0,"Estoque Negativo",tbResumo[[#This Row],[Saldo Atual]]=0,"Obsoleto",tbResumo[[#This Row],[Saldo Atual]]&lt;=20,"Crítico",tbResumo[[#This Row],[Saldo Atual]]&lt;=100,"OK",tbResumo[[#This Row],[Saldo Atual]]&gt;100,"Excesso")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9165,7 +9268,7 @@
     <col min="1" max="1" width="15.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" customWidth="1"/>
     <col min="3" max="3" width="28.88671875" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="21.44140625" customWidth="1"/>
     <col min="6" max="6" width="26.109375" customWidth="1"/>
   </cols>
@@ -9180,7 +9283,7 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>67</v>
       </c>
       <c r="E1" t="s">
@@ -9201,7 +9304,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <v>80</v>
       </c>
       <c r="E2" t="s">
@@ -9222,7 +9325,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Caixa de Som MiniBass</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <v>60</v>
       </c>
       <c r="E3" t="s">
@@ -9243,7 +9346,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>100</v>
       </c>
       <c r="E4" t="s">
@@ -9264,7 +9367,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Teclado Mecânico KeyStorm</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>45</v>
       </c>
       <c r="E5" t="s">
@@ -9285,7 +9388,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Webcam Full HD VisionCam</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>50</v>
       </c>
       <c r="E6" t="s">
@@ -9306,7 +9409,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>120</v>
       </c>
       <c r="E7" t="s">
@@ -9327,7 +9430,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>200</v>
       </c>
       <c r="E8" t="s">
@@ -9348,7 +9451,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>70</v>
       </c>
       <c r="E9" t="s">
@@ -9369,7 +9472,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>40</v>
       </c>
       <c r="E10" t="s">
@@ -9390,7 +9493,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>65</v>
       </c>
       <c r="E11" t="s">
@@ -9411,7 +9514,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>55</v>
       </c>
       <c r="E12" t="s">
@@ -9432,7 +9535,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>75</v>
       </c>
       <c r="E13" t="s">
@@ -9453,7 +9556,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>90</v>
       </c>
       <c r="E14" t="s">
@@ -9474,7 +9577,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>150</v>
       </c>
       <c r="E15" t="s">
@@ -9495,7 +9598,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <v>110</v>
       </c>
       <c r="E16" t="s">
@@ -9516,7 +9619,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>30</v>
       </c>
       <c r="E17" t="s">
@@ -9537,7 +9640,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>50</v>
       </c>
       <c r="E18" t="s">
@@ -9558,7 +9661,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
         <v>100</v>
       </c>
       <c r="E19" t="s">
@@ -9579,7 +9682,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
         <v>40</v>
       </c>
       <c r="E20" t="s">
@@ -9600,7 +9703,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>80</v>
       </c>
       <c r="E21" t="s">
@@ -9621,7 +9724,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
         <v>35</v>
       </c>
       <c r="E22" t="s">
@@ -9642,7 +9745,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="4">
         <v>25</v>
       </c>
       <c r="E23" t="s">
@@ -9663,7 +9766,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="4">
         <v>30</v>
       </c>
       <c r="E24" t="s">
@@ -9684,7 +9787,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="4">
         <v>45</v>
       </c>
       <c r="E25" t="s">
@@ -9705,7 +9808,7 @@
         <f>_xlfn.XLOOKUP(tbEntrada[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="4">
         <v>20</v>
       </c>
       <c r="E26" t="s">
@@ -9731,7 +9834,7 @@
     <col min="1" max="1" width="16.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" customWidth="1"/>
     <col min="3" max="3" width="20.5546875" customWidth="1"/>
-    <col min="4" max="4" width="26.44140625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="26.44140625" style="4" customWidth="1"/>
     <col min="5" max="5" width="24.21875" customWidth="1"/>
     <col min="6" max="6" width="26.44140625" customWidth="1"/>
   </cols>
@@ -9746,7 +9849,7 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>75</v>
       </c>
       <c r="E1" t="s">
@@ -9766,7 +9869,7 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <v>12</v>
       </c>
       <c r="E2" t="s">
@@ -9786,7 +9889,7 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <v>8</v>
       </c>
       <c r="E3" t="s">
@@ -9806,7 +9909,7 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>20</v>
       </c>
       <c r="E4" t="s">
@@ -9826,7 +9929,7 @@
       <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>10</v>
       </c>
       <c r="E5" t="s">
@@ -9846,7 +9949,7 @@
       <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>15</v>
       </c>
       <c r="E6" t="s">
@@ -9866,7 +9969,7 @@
       <c r="C7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>35</v>
       </c>
       <c r="E7" t="s">
@@ -9887,7 +9990,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>70</v>
       </c>
       <c r="E8" t="s">
@@ -9908,7 +10011,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>18</v>
       </c>
       <c r="E9" t="s">
@@ -9929,7 +10032,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>9</v>
       </c>
       <c r="E10" t="s">
@@ -9950,7 +10053,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>16</v>
       </c>
       <c r="E11" t="s">
@@ -9971,7 +10074,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>14</v>
       </c>
       <c r="E12" t="s">
@@ -9992,7 +10095,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>22</v>
       </c>
       <c r="E13" t="s">
@@ -10013,7 +10116,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>30</v>
       </c>
       <c r="E14" t="s">
@@ -10034,7 +10137,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>60</v>
       </c>
       <c r="E15" t="s">
@@ -10055,7 +10158,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <v>28</v>
       </c>
       <c r="E16" t="s">
@@ -10076,7 +10179,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Fone Bluetooth AirMax</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>25</v>
       </c>
       <c r="E17" t="s">
@@ -10097,7 +10200,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Mouse Gamer ProClick</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>32</v>
       </c>
       <c r="E18" t="s">
@@ -10118,7 +10221,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Carregador USB-C Turbo</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
         <v>48</v>
       </c>
       <c r="E19" t="s">
@@ -10139,7 +10242,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Cabo USB-C Reforçado</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
         <v>95</v>
       </c>
       <c r="E20" t="s">
@@ -10160,7 +10263,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>SSD 480GB FastDisk</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>42</v>
       </c>
       <c r="E21" t="s">
@@ -10181,7 +10284,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Pendrive 64GB DataGo</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
         <v>110</v>
       </c>
       <c r="E22" t="s">
@@ -10202,7 +10305,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Tomada Inteligente Wi-Fi</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="4">
         <v>20</v>
       </c>
       <c r="E23" t="s">
@@ -10223,7 +10326,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Repetidor de Sinal Wi-Fi</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="4">
         <v>35</v>
       </c>
       <c r="E24" t="s">
@@ -10244,7 +10347,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Hub USB 4 Portas</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="4">
         <v>50</v>
       </c>
       <c r="E25" t="s">
@@ -10265,7 +10368,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Caixa de Som MiniBass</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="4">
         <v>18</v>
       </c>
       <c r="E26" t="s">
@@ -10286,7 +10389,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Teclado Mecânico KeyStorm</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="4">
         <v>22</v>
       </c>
       <c r="E27" t="s">
@@ -10307,7 +10410,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Webcam Full HD VisionCam</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="4">
         <v>25</v>
       </c>
       <c r="E28" t="s">
@@ -10328,7 +10431,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Power Bank 10000mAh</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="4">
         <v>40</v>
       </c>
       <c r="E29" t="s">
@@ -10349,7 +10452,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Luminária LED Smart</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="4">
         <v>18</v>
       </c>
       <c r="E30" t="s">
@@ -10370,7 +10473,7 @@
         <f>_xlfn.XLOOKUP(tbSaida[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Produto],"SKU não encontrado")</f>
         <v>Roteador Wi-Fi Dual Band</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="4">
         <v>26</v>
       </c>
       <c r="E31" t="s">
@@ -10398,10 +10501,10 @@
   <cols>
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
     <col min="3" max="3" width="26.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" style="5" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" style="4" customWidth="1"/>
     <col min="8" max="8" width="25.109375" customWidth="1"/>
     <col min="9" max="9" width="18.44140625" customWidth="1"/>
   </cols>
@@ -10416,16 +10519,16 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>84</v>
       </c>
       <c r="H1" t="s">
@@ -10447,23 +10550,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Áudio</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>129.9</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>110</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>37</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>73</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>9482.7000000000007</v>
       </c>
@@ -10484,23 +10587,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Áudio</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>89.9</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>60</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>26</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>34</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>3056.6000000000004</v>
       </c>
@@ -10521,23 +10624,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>79.900000000000006</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>135</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>52</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>83</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>6631.7000000000007</v>
       </c>
@@ -10558,23 +10661,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>219.9</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>45</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>32</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>13</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2858.7000000000003</v>
       </c>
@@ -10595,23 +10698,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Periféricos</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>159.9</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>50</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>10</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>1599</v>
       </c>
@@ -10632,23 +10735,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>69.900000000000006</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>170</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>83</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>87</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>6081.3</v>
       </c>
@@ -10669,23 +10772,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>29.9</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>300</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>165</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>135</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>4036.5</v>
       </c>
@@ -10706,23 +10809,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>119.9</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>90</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>58</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>32</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>3836.8</v>
       </c>
@@ -10743,23 +10846,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Casa Inteligente</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>149.9</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>27</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>13</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>1948.7</v>
       </c>
@@ -10780,23 +10883,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Casa Inteligente</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>99.9</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>90</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>36</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>54</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>5394.6</v>
       </c>
@@ -10817,23 +10920,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Redes</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>189.9</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>55</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>40</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>15</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2848.5</v>
       </c>
@@ -10854,23 +10957,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Redes</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>109.9</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>105</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>57</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>48</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>5275.2000000000007</v>
       </c>
@@ -10891,23 +10994,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Armazenamento</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>259.89999999999998</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>130</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>72</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>58</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>15074.199999999999</v>
       </c>
@@ -10928,23 +11031,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Armazenamento</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>49.9</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>230</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>170</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>60</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>2994</v>
       </c>
@@ -10965,23 +11068,23 @@
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Categoria],"Não encontrado")</f>
         <v>Acessórios</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="5">
         <f>_xlfn.XLOOKUP(tbResumo[[#This Row],[SKU]],tbCadastro[SKU],tbCadastro[Preço Unitário],0)</f>
         <v>59.9</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <f>SUMIFS(tbEntrada[Quantidade Entrada],tbEntrada[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>155</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <f>SUMIFS(tbSaida[Quantidade Saída],tbSaida[SKU],tbResumo[[#This Row],[SKU]])</f>
         <v>78</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="4">
         <f>tbResumo[[#This Row],[Total Entradas]]-tbResumo[[#This Row],[Total Saídas]]</f>
         <v>77</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="5">
         <f>tbResumo[[#This Row],[Saldo Atual]]*tbResumo[[#This Row],[Preço Unitário]]</f>
         <v>4612.3</v>
       </c>
@@ -10991,40 +11094,20 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I1048576">
-    <cfRule type="containsText" dxfId="9" priority="11" operator="containsText" text="Estoque Negativo">
-      <formula>NOT(ISERROR(SEARCH("Estoque Negativo",I2)))</formula>
+  <conditionalFormatting sqref="G2:G1048576">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="between">
+      <formula>21</formula>
+      <formula>99</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="Obsoleto">
-      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="greaterThan">
+      <formula>100</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="Obsoleto">
-      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="Crítico">
-      <formula>NOT(ISERROR(SEARCH("Crítico",I2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="OK">
-      <formula>NOT(ISERROR(SEARCH("OK",I2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="Excesso">
-      <formula>NOT(ISERROR(SEARCH("Excesso",I2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="between">
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="between">
       <formula>1</formula>
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
-      <formula>100</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="between">
-      <formula>21</formula>
-      <formula>99</formula>
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H1048576">
@@ -11039,6 +11122,26 @@
           <x14:id>{C20CB109-B948-4D59-A50C-2622DC3F61EC}</x14:id>
         </ext>
       </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I1048576">
+    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="Excesso">
+      <formula>NOT(ISERROR(SEARCH("Excesso",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="OK">
+      <formula>NOT(ISERROR(SEARCH("OK",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="8" operator="containsText" text="Crítico">
+      <formula>NOT(ISERROR(SEARCH("Crítico",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="9" operator="containsText" text="Obsoleto">
+      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="10" operator="containsText" text="Obsoleto">
+      <formula>NOT(ISERROR(SEARCH("Obsoleto",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="11" operator="containsText" text="Estoque Negativo">
+      <formula>NOT(ISERROR(SEARCH("Estoque Negativo",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -11095,25 +11198,25 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>87</v>
       </c>
       <c r="B3" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>87</v>
       </c>
       <c r="E3" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>87</v>
       </c>
       <c r="H3" t="s">
         <v>93</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="6" t="s">
         <v>87</v>
       </c>
       <c r="K3" t="s">
@@ -11121,184 +11224,184 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>18566.899999999998</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4">
         <v>4</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>69.900000000000006</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <v>715</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <v>18068.199999999997</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5">
         <v>2</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <v>154.89999999999998</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>360</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <v>12539.300000000001</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6">
         <v>2</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <v>109.9</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <v>7343.3</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7">
         <v>2</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <v>124.9</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <v>11089.400000000001</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8">
         <v>3</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <v>153.23333333333335</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="5">
         <v>8123.7000000000007</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9">
         <v>2</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="5">
         <v>149.9</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="5">
         <v>75730.8</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10">
         <v>15</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="5">
         <v>121.23333333333336</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <v>1765</v>
       </c>
     </row>
@@ -11306,18 +11409,18 @@
       <c r="A13" t="s">
         <v>100</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>87</v>
       </c>
       <c r="B15" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>87</v>
       </c>
       <c r="E15" t="s">
@@ -11325,154 +11428,154 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16">
         <v>4</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="5">
         <v>15074.199999999999</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17">
         <v>1</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="5">
         <v>9482.7000000000007</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18">
         <v>10</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="5">
         <v>6631.7000000000007</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19">
         <v>15</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="5">
         <v>6081.3</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="5">
         <v>5394.6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="5">
         <v>5275.2000000000007</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="5">
         <v>4612.3</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <v>4036.5</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="5">
         <v>3836.8</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <v>3056.6000000000004</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="5">
         <v>2994</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="5">
         <v>2858.7000000000003</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="5">
         <v>2848.5</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="5">
         <v>1948.7</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="5">
         <v>1599</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="5">
         <v>75730.8</v>
       </c>
     </row>
@@ -11483,9 +11586,82 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65D9A2C6-B7C6-4CED-BE71-2DF0E82A99A1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="7.5546875" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="17" max="17" width="23.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="A1" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+    </row>
+    <row r="3" spans="1:15" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="19"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="I3" s="12"/>
+      <c r="J3" s="13"/>
+      <c r="L3" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="13"/>
+    </row>
+    <row r="4" spans="1:15" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="A4" s="17">
+        <f>SUM(tbResumo[Valor em Estoque])</f>
+        <v>75730.8</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="15"/>
+      <c r="E4" s="20">
+        <f>COUNTA(tbResumo[SKU])</f>
+        <v>15</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="H4" s="21">
+        <f>COUNTIF(tbResumo[Status do Produto],"Crítico")</f>
+        <v>4</v>
+      </c>
+      <c r="I4" s="14"/>
+      <c r="J4" s="15"/>
+      <c r="L4" s="21">
+        <f>COUNTIF(tbResumo[Status do Produto],"Excesso")</f>
+        <v>1</v>
+      </c>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="15"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>